<commit_message>
Fix ruby xlsx restoration alignment
Co-authored-by: Linden10 <20895359+Linden10@users.noreply.github.com>
Agent-Logs-Url: https://github.com/Linden10/misc_game-chs/sessions/381ba50c-f050-426c-8d85-93a0bd2c9f49
</commit_message>
<xml_diff>
--- a/processed_ruby_restored_xlsx/sc013_１日目添い寝.ss.xlsx
+++ b/processed_ruby_restored_xlsx/sc013_１日目添い寝.ss.xlsx
@@ -547,8 +547,8 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>In the end I couldn't tell who wrote it, but somehow I
-have a feeling about everyone.</t>
+          <t>In the end I couldn't tell who wrote it, but somehow
+I have a feeling about everyone.</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -582,8 +582,8 @@
         <is>
           <t>If we're talking pure clinginess then Rurichiyo-chan
 fits too, and Nono-chan just arrived on this
-island—she might be anxious even if she hasn't said it
-out loud.</t>
+island—she might be anxious even if she hasn't said
+it out loud.</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -629,8 +629,8 @@
       <c r="B11" s="1" t="inlineStr">
         <is>
           <t>They probably couldn't say it there with the others
-around, but they were also questioned about who they'd
-sleep beside.</t>
+around, but they were also questioned about who
+they'd sleep beside.</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -814,8 +814,8 @@
       <c r="B23" s="1" t="inlineStr">
         <is>
           <t>She's the type who most innocently would have written
-it, and imagining that Miru-chan really did is just so
-cute.</t>
+it, and imagining that Miru-chan really did is just
+so cute.</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -830,9 +830,9 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>Besides, she'd probably accept without hesitation, and
-it seems like we'd get to have a cuddly sleep beside
-her......</t>
+          <t>Besides, she'd probably accept without hesitation,
+and it seems like we'd get to have a cuddly sleep
+beside her......</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -972,8 +972,8 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>The lights are out, and it looks like both of them are
-already asleep.</t>
+          <t>The lights are out, and it looks like both of them
+are already asleep.</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1282,7 +1282,8 @@
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>She probably felt the draft when I lifted the blanket.</t>
+          <t>She probably felt the draft when I lifted the
+blanket.</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -1327,8 +1328,8 @@
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
-          <t>...Once the futon warms up, her breathing goes back to
-normal.</t>
+          <t>...Once the futon warms up, her breathing goes back
+to normal.</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1463,9 +1464,9 @@
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>Even asleep, if she reacts just to the temperature she
-feels, then... what would happen if I touched her with
-my hand？</t>
+          <t>Even asleep, if she reacts just to the temperature
+she feels, then... what would happen if I touched her
+with my hand？</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -1481,8 +1482,8 @@
       <c r="B66" s="1" t="inlineStr">
         <is>
           <t>Usually Miru-chan comes over to me, but when she does
-that her mood comes first, so sensation probably takes
-a backseat.</t>
+that her mood comes first, so sensation probably
+takes a backseat.</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -1497,8 +1498,8 @@
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>But now, unconscious and defenseless, Miru-chan's true
-sensitivity should be completely exposed.</t>
+          <t>But now, unconscious and defenseless, Miru-chan's
+true sensitivity should be completely exposed.</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -1573,8 +1574,8 @@
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t>I won't allow that expression to be distorted even for
-an instant...！</t>
+          <t>I won't allow that expression to be distorted even
+for an instant...！</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -2104,7 +2105,8 @@
       </c>
       <c r="B107" s="1" t="inlineStr">
         <is>
-          <t>When I left her alone, this time she started laughing.</t>
+          <t>When I left her alone, this time she started
+laughing.</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -2134,7 +2136,8 @@
       </c>
       <c r="B109" s="1" t="inlineStr">
         <is>
-          <t>Maybe she's dreaming about roughhousing with everyone？</t>
+          <t>Maybe she's dreaming about roughhousing with
+everyone？</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -2335,8 +2338,8 @@
       </c>
       <c r="B122" s="1" t="inlineStr">
         <is>
-          <t>...Miru-chan started sucking on the finger I’d pressed
-to her lips！</t>
+          <t>...Miru-chan started sucking on the finger I’d
+pressed to her lips！</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -2566,7 +2569,8 @@
       <c r="B137" s="1" t="inlineStr">
         <is>
           <t>Maybe because she was sucking in her sleep, she
-couldn’t breathe properly between breaths... probably.</t>
+couldn’t breathe properly between breaths...
+probably.</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -2596,8 +2600,8 @@
       </c>
       <c r="B139" s="1" t="inlineStr">
         <is>
-          <t>After all, today’s sex-ed should have been stimulating
-for Miru-chan too.</t>
+          <t>After all, today’s sex-ed should have been
+stimulating for Miru-chan too.</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -3375,9 +3379,9 @@
       </c>
       <c r="B190" s="1" t="inlineStr">
         <is>
-          <t>Because she was asleep, it was probably harder for her
-to exhale, but there was also the thing earlier where
-she latched onto my finger.</t>
+          <t>Because she was asleep, it was probably harder for
+her to exhale, but there was also the thing earlier
+where she latched onto my finger.</t>
         </is>
       </c>
       <c r="C190" t="n">
@@ -3636,8 +3640,8 @@
       </c>
       <c r="B207" s="1" t="inlineStr">
         <is>
-          <t>I tried to pull my tongue back during that moment, but
-I became unable to move.</t>
+          <t>I tried to pull my tongue back during that moment,
+but I became unable to move.</t>
         </is>
       </c>
       <c r="C207" t="n">
@@ -3667,8 +3671,8 @@
       </c>
       <c r="B209" s="1" t="inlineStr">
         <is>
-          <t>Our saliva, glinting, stretching into a string between
-her upper and lower lips…</t>
+          <t>Our saliva, glinting, stretching into a string
+between her upper and lower lips…</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -4446,8 +4450,8 @@
       </c>
       <c r="B260" s="1" t="inlineStr">
         <is>
-          <t>When I pulled my face away without thinking, Miru-chan
-smiled satisﬁedly.</t>
+          <t>When I pulled my face away without thinking,
+Miru-chan smiled satisﬁedly.</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -4478,7 +4482,8 @@
       </c>
       <c r="B262" s="1" t="inlineStr">
         <is>
-          <t>No, rather, I should say I was led to it by Miru-chan…</t>
+          <t>No, rather, I should say I was led to it by
+Miru-chan…</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -4493,7 +4498,8 @@
       </c>
       <c r="B263" s="1" t="inlineStr">
         <is>
-          <t>Against a sleeping Miru-chan, I'm completely helpless.</t>
+          <t>Against a sleeping Miru-chan, I'm completely
+helpless.</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -4554,8 +4560,9 @@
       </c>
       <c r="B267" s="1" t="inlineStr">
         <is>
-          <t>Earlier she was responding in her sleep to my teasing,
-but now it feels like she's drifted into a deep sleep.</t>
+          <t>Earlier she was responding in her sleep to my
+teasing, but now it feels like she's drifted into a
+deep sleep.</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -4679,8 +4686,8 @@
       </c>
       <c r="B275" s="1" t="inlineStr">
         <is>
-          <t>Contrary to her usual sassy attitude, she's actually a
-shy, somewhat socially awkward, and kind of lonely
+          <t>Contrary to her usual sassy attitude, she's actually
+a shy, somewhat socially awkward, and kind of lonely
 girl...</t>
         </is>
       </c>
@@ -5144,8 +5151,8 @@
       </c>
       <c r="B305" s="1" t="inlineStr">
         <is>
-          <t>Rin-chan's sleeping face can be summed up in one word:
-cute.</t>
+          <t>Rin-chan's sleeping face can be summed up in one
+word: cute.</t>
         </is>
       </c>
       <c r="C305" t="n">
@@ -5191,8 +5198,8 @@
       <c r="B308" s="1" t="inlineStr">
         <is>
           <t>She’s usually cheeky and sharp-tongued, messing me
-about, but she can be shy and easily frightened, which
-is kind of cute.</t>
+about, but she can be shy and easily frightened,
+which is kind of cute.</t>
         </is>
       </c>
       <c r="C308" t="n">
@@ -5254,8 +5261,8 @@
       </c>
       <c r="B312" s="1" t="inlineStr">
         <is>
-          <t>I couldn't even go so far as to play a prank on her as
-payback...</t>
+          <t>I couldn't even go so far as to play a prank on her
+as payback...</t>
         </is>
       </c>
       <c r="C312" t="n">
@@ -5331,7 +5338,8 @@
       </c>
       <c r="B317" s="1" t="inlineStr">
         <is>
-          <t>It was as if she were embarrassed at catching my gaze.</t>
+          <t>It was as if she were embarrassed at catching my
+gaze.</t>
         </is>
       </c>
       <c r="C317" t="n">
@@ -5363,8 +5371,8 @@
       <c r="B319" s="1" t="inlineStr">
         <is>
           <t>...But Rin-chan has that kind of quick intuition that
-makes me think she might, and that's one of the things
-that teases me.</t>
+makes me think she might, and that's one of the
+things that teases me.</t>
         </is>
       </c>
       <c r="C319" t="n">
@@ -5471,8 +5479,8 @@
       </c>
       <c r="B326" s="1" t="inlineStr">
         <is>
-          <t>Right now, she probably wouldn't notice no matter what
-I did.</t>
+          <t>Right now, she probably wouldn't notice no matter
+what I did.</t>
         </is>
       </c>
       <c r="C326" t="n">
@@ -5657,8 +5665,8 @@
       </c>
       <c r="B338" s="1" t="inlineStr">
         <is>
-          <t>...It's such a trivial thing, but it weirdly turned me
-on.</t>
+          <t>...It's such a trivial thing, but it weirdly turned
+me on.</t>
         </is>
       </c>
       <c r="C338" t="n">
@@ -5688,8 +5696,8 @@
       </c>
       <c r="B340" s="1" t="inlineStr">
         <is>
-          <t>No, that's not it. These half-open lips are those of a
-girl waiting for a kiss...！</t>
+          <t>No, that's not it. These half-open lips are those of
+a girl waiting for a kiss...！</t>
         </is>
       </c>
       <c r="C340" t="n">
@@ -5827,7 +5835,8 @@
       </c>
       <c r="B349" s="1" t="inlineStr">
         <is>
-          <t>Uwaa... just thinking about it makes my heart race...！</t>
+          <t>Uwaa... just thinking about it makes my heart
+race...！</t>
         </is>
       </c>
       <c r="C349" t="n">
@@ -6619,8 +6628,8 @@
       </c>
       <c r="B401" s="1" t="inlineStr">
         <is>
-          <t>Normally, Rin-chan is quick with words when it counts,
-so it's scary when she doesn't speak.</t>
+          <t>Normally, Rin-chan is quick with words when it
+counts, so it's scary when she doesn't speak.</t>
         </is>
       </c>
       <c r="C401" t="n">
@@ -6846,8 +6855,8 @@
       </c>
       <c r="B416" s="1" t="inlineStr">
         <is>
-          <t>Her face is still red, but Rin-chan's usual expression
-is back.</t>
+          <t>Her face is still red, but Rin-chan's usual
+expression is back.</t>
         </is>
       </c>
       <c r="C416" t="n">
@@ -7607,8 +7616,8 @@
       </c>
       <c r="B466" s="1" t="inlineStr">
         <is>
-          <t>She wanted to see a hidden act somewhere away from the
-others.</t>
+          <t>She wanted to see a hidden act somewhere away from
+the others.</t>
         </is>
       </c>
       <c r="C466" t="n">
@@ -7775,9 +7784,9 @@
       </c>
       <c r="B477" s="1" t="inlineStr">
         <is>
-          <t>Rin-chan, who didn't know what 'okazu' meant, frowned,
-thinking she'd been told something completely
-unrelated.</t>
+          <t>Rin-chan, who didn't know what 'okazu' meant,
+frowned, thinking she'd been told something
+completely unrelated.</t>
         </is>
       </c>
       <c r="C477" t="n">
@@ -8312,8 +8321,8 @@
       <c r="B512" s="1" t="inlineStr">
         <is>
           <t>The fact she handed me her panties probably meant yes
-to that sort of thing, but when push came to shove she
-might get so embarrassed she’d start to cry.</t>
+to that sort of thing, but when push came to shove
+she might get so embarrassed she’d start to cry.</t>
         </is>
       </c>
       <c r="C512" t="n">
@@ -8560,8 +8569,8 @@
       </c>
       <c r="B528" s="1" t="inlineStr">
         <is>
-          <t>Rin-chan said in a slightly annoyed voice, hugging her
-knees with a faintly troubled expression.</t>
+          <t>Rin-chan said in a slightly annoyed voice, hugging
+her knees with a faintly troubled expression.</t>
         </is>
       </c>
       <c r="C528" t="n">
@@ -9086,8 +9095,8 @@
       </c>
       <c r="B562" s="1" t="inlineStr">
         <is>
-          <t>A warm, reassuring sense of being enveloped...or so to
-speak.</t>
+          <t>A warm, reassuring sense of being enveloped...or so
+to speak.</t>
         </is>
       </c>
       <c r="C562" t="n">
@@ -9102,9 +9111,9 @@
       </c>
       <c r="B563" s="1" t="inlineStr">
         <is>
-          <t>But the parent bird's feathers are unexpectedly stiff,
-and there's a sternness to them that pushes the chick
-to fly off sooner.</t>
+          <t>But the parent bird's feathers are unexpectedly
+stiff, and there's a sternness to them that pushes
+the chick to fly off sooner.</t>
         </is>
       </c>
       <c r="C563" t="n">
@@ -9427,8 +9436,8 @@
       </c>
       <c r="B584" s="1" t="inlineStr">
         <is>
-          <t>When I stopped and my mind started working, I realized
-I was doing something really embarrassing...</t>
+          <t>When I stopped and my mind started working, I
+realized I was doing something really embarrassing...</t>
         </is>
       </c>
       <c r="C584" t="n">
@@ -9565,8 +9574,8 @@
       </c>
       <c r="B593" s="1" t="inlineStr">
         <is>
-          <t>When I look straight ahead, Rin-chan's cute slit comes
-into view.</t>
+          <t>When I look straight ahead, Rin-chan's cute slit
+comes into view.</t>
         </is>
       </c>
       <c r="C593" t="n">
@@ -9672,8 +9681,8 @@
       </c>
       <c r="B600" s="1" t="inlineStr">
         <is>
-          <t>From the patterns observed so far, that’s a sign she’s
-embarrassed.</t>
+          <t>From the patterns observed so far, that’s a sign
+she’s embarrassed.</t>
         </is>
       </c>
       <c r="C600" t="n">
@@ -9918,7 +9927,8 @@
       <c r="B616" s="1" t="inlineStr">
         <is>
           <t>While she fidgeted, her butt would drop and that area
-would become harder to see, but that’s also an accent.</t>
+would become harder to see, but that’s also an
+accent.</t>
         </is>
       </c>
       <c r="C616" t="n">
@@ -10133,8 +10143,8 @@
       </c>
       <c r="B630" s="1" t="inlineStr">
         <is>
-          <t>「Ahh... the stuff coming out from the tip's getting on
-the panties...」</t>
+          <t>「Ahh... the stuff coming out from the tip's getting
+on the panties...」</t>
         </is>
       </c>
       <c r="C630" t="n">
@@ -10407,8 +10417,8 @@
       </c>
       <c r="B648" s="1" t="inlineStr">
         <is>
-          <t>I meant to respond sincerely, but Rin-chan widened her
-eyes like it was the first she'd heard of it.</t>
+          <t>I meant to respond sincerely, but Rin-chan widened
+her eyes like it was the first she'd heard of it.</t>
         </is>
       </c>
       <c r="C648" t="n">
@@ -10532,8 +10542,8 @@
       </c>
       <c r="B656" s="1" t="inlineStr">
         <is>
-          <t>Ah, this mix of shame and bewilderment is irresistible
-too！</t>
+          <t>Ah, this mix of shame and bewilderment is
+irresistible too！</t>
         </is>
       </c>
       <c r="C656" t="n">
@@ -10807,9 +10817,9 @@
       </c>
       <c r="B674" s="1" t="inlineStr">
         <is>
-          <t>She's a little desperate and still looks troubled, but
-the light in her eyes is slowly returning to the usual
-Rin-chan.</t>
+          <t>She's a little desperate and still looks troubled,
+but the light in her eyes is slowly returning to the
+usual Rin-chan.</t>
         </is>
       </c>
       <c r="C674" t="n">
@@ -10841,8 +10851,8 @@
       <c r="B676" s="1" t="inlineStr">
         <is>
           <t>Feeling that again, I turned my hips toward Rin-chan
-once more and began stroking myself toward ejaculation
-however I liked.</t>
+once more and began stroking myself toward
+ejaculation however I liked.</t>
         </is>
       </c>
       <c r="C676" t="n">
@@ -11069,8 +11079,8 @@
       </c>
       <c r="B691" s="1" t="inlineStr">
         <is>
-          <t>「Right... and once it gets used to it, gradually speed
-up.」</t>
+          <t>「Right... and once it gets used to it, gradually
+speed up.」</t>
         </is>
       </c>
       <c r="C691" t="n">
@@ -11223,8 +11233,8 @@
       </c>
       <c r="B701" s="1" t="inlineStr">
         <is>
-          <t>When I stroked my penis at high speed, Rin-chan opened
-her eyes and mouth wide.</t>
+          <t>When I stroked my penis at high speed, Rin-chan
+opened her eyes and mouth wide.</t>
         </is>
       </c>
       <c r="C701" t="n">
@@ -11561,8 +11571,8 @@
       </c>
       <c r="B723" s="1" t="inlineStr">
         <is>
-          <t>Sensing my strange presence, Rin-chan called out to me
-with concern.</t>
+          <t>Sensing my strange presence, Rin-chan called out to
+me with concern.</t>
         </is>
       </c>
       <c r="C723" t="n">
@@ -11836,8 +11846,8 @@
       </c>
       <c r="B741" s="1" t="inlineStr">
         <is>
-          <t>The spurting semen arced through the air, and Rin-chan
-let out a small cry.</t>
+          <t>The spurting semen arced through the air, and
+Rin-chan let out a small cry.</t>
         </is>
       </c>
       <c r="C741" t="n">
@@ -12005,8 +12015,8 @@
       </c>
       <c r="B752" s="1" t="inlineStr">
         <is>
-          <t>It's like embarrassment has reached its absolute limit
-here...</t>
+          <t>It's like embarrassment has reached its absolute
+limit here...</t>
         </is>
       </c>
       <c r="C752" t="n">
@@ -12021,8 +12031,8 @@
       </c>
       <c r="B753" s="1" t="inlineStr">
         <is>
-          <t>It's better than her emotions exploding into a scream,
-but with Rin-chan it's scary from here on.</t>
+          <t>It's better than her emotions exploding into a
+scream, but with Rin-chan it's scary from here on.</t>
         </is>
       </c>
       <c r="C753" t="n">
@@ -12038,7 +12048,8 @@
       <c r="B754" s="1" t="inlineStr">
         <is>
           <t>I braced myself to be scolded, and while Rin-chan
-stayed frozen I quickly put on my underwear and pants.</t>
+stayed frozen I quickly put on my underwear and
+pants.</t>
         </is>
       </c>
       <c r="C754" t="n">
@@ -12420,9 +12431,9 @@
       </c>
       <c r="B779" s="1" t="inlineStr">
         <is>
-          <t>Semen was still between her legs, but she was probably
-so angry she didn’t even care about something like
-that.</t>
+          <t>Semen was still between her legs, but she was
+probably so angry she didn’t even care about
+something like that.</t>
         </is>
       </c>
       <c r="C779" t="n">
@@ -12467,8 +12478,8 @@
       </c>
       <c r="B782" s="1" t="inlineStr">
         <is>
-          <t>「...But you said 'show me,' Rin, so... I guess I can't
-really blame you...」</t>
+          <t>「...But you said 'show me,' Rin, so... I guess I
+can't really blame you...」</t>
         </is>
       </c>
       <c r="C782" t="n">
@@ -12729,8 +12740,8 @@
       </c>
       <c r="B799" s="1" t="inlineStr">
         <is>
-          <t>Rin-chan spoke in a soft voice, then turned to me with
-a face like she was about to cry.</t>
+          <t>Rin-chan spoke in a soft voice, then turned to me
+with a face like she was about to cry.</t>
         </is>
       </c>
       <c r="C799" t="n">
@@ -12979,8 +12990,8 @@
       </c>
       <c r="B815" s="1" t="inlineStr">
         <is>
-          <t>It was then I realized I was still gripping Rin-chan's
-panties.</t>
+          <t>It was then I realized I was still gripping
+Rin-chan's panties.</t>
         </is>
       </c>
       <c r="C815" t="n">
@@ -13090,8 +13101,8 @@
         <is>
           <t>Normally she ends up playing the sensible one, so she
 looks the most mature among everyone, but when she
-wants attention, Rurichiyo-chan is the least shy about
-it.</t>
+wants attention, Rurichiyo-chan is the least shy
+about it.</t>
         </is>
       </c>
       <c r="C822" t="n">
@@ -13121,8 +13132,9 @@
       </c>
       <c r="B824" s="1" t="inlineStr">
         <is>
-          <t>Sometimes she's the one being coddled, sometimes she's
-the one who spoils me, and it always soothes my heart.</t>
+          <t>Sometimes she's the one being coddled, sometimes
+she's the one who spoils me, and it always soothes my
+heart.</t>
         </is>
       </c>
       <c r="C824" t="n">
@@ -13169,8 +13181,8 @@
       <c r="B827" s="1" t="inlineStr">
         <is>
           <t>There's a closeness that comes from being uncle and
-niece, sure, but I feel something between us that goes
-beyond that relationship.</t>
+niece, sure, but I feel something between us that
+goes beyond that relationship.</t>
         </is>
       </c>
       <c r="C827" t="n">
@@ -13230,8 +13242,8 @@
       </c>
       <c r="B831" s="1" t="inlineStr">
         <is>
-          <t>Ah... this is Rurichiyo-chan and Nono-chan's room now,
-huh.</t>
+          <t>Ah... this is Rurichiyo-chan and Nono-chan's room
+now, huh.</t>
         </is>
       </c>
       <c r="C831" t="n">
@@ -13310,8 +13322,8 @@
       </c>
       <c r="B836" s="1" t="inlineStr">
         <is>
-          <t>I peered in from below, and luckily Rurichiyo-chan was
-in the lower bunk.</t>
+          <t>I peered in from below, and luckily Rurichiyo-chan
+was in the lower bunk.</t>
         </is>
       </c>
       <c r="C836" t="n">
@@ -13371,8 +13383,8 @@
       </c>
       <c r="B840" s="1" t="inlineStr">
         <is>
-          <t>Maybe she sensed me — Rurichiyo-chan opened her eyes a
-little and sat up with a groggy start.</t>
+          <t>Maybe she sensed me — Rurichiyo-chan opened her eyes
+a little and sat up with a groggy start.</t>
         </is>
       </c>
       <c r="C840" t="n">
@@ -13828,7 +13840,8 @@
       </c>
       <c r="B870" s="1" t="inlineStr">
         <is>
-          <t>Rurichiyo-chan fell back onto the bed holding my head.</t>
+          <t>Rurichiyo-chan fell back onto the bed holding my
+head.</t>
         </is>
       </c>
       <c r="C870" t="n">
@@ -14015,8 +14028,8 @@
       </c>
       <c r="B882" s="1" t="inlineStr">
         <is>
-          <t>Being held like this, with my head trapped, is kind of
-wonderful, but I can’t do anything like this.</t>
+          <t>Being held like this, with my head trapped, is kind
+of wonderful, but I can’t do anything like this.</t>
         </is>
       </c>
       <c r="C882" t="n">
@@ -14570,7 +14583,8 @@
       </c>
       <c r="B918" s="1" t="inlineStr">
         <is>
-          <t>Is Rurichiyo-chan dreaming that she's soothing a baby？</t>
+          <t>Is Rurichiyo-chan dreaming that she's soothing a
+baby？</t>
         </is>
       </c>
       <c r="C918" t="n">
@@ -14862,7 +14876,8 @@
       </c>
       <c r="B937" s="1" t="inlineStr">
         <is>
-          <t>Rurichiyo-chan starts unbuttoning her pajamas herself.</t>
+          <t>Rurichiyo-chan starts unbuttoning her pajamas
+herself.</t>
         </is>
       </c>
       <c r="C937" t="n">
@@ -14877,9 +14892,9 @@
       </c>
       <c r="B938" s="1" t="inlineStr">
         <is>
-          <t>I pretty much knew what kind of dream you were having,
-but to go this far — what a child so full of maternal
-instinct...！</t>
+          <t>I pretty much knew what kind of dream you were
+having, but to go this far — what a child so full of
+maternal instinct...！</t>
         </is>
       </c>
       <c r="C938" t="n">
@@ -15033,8 +15048,8 @@
       </c>
       <c r="B948" s="1" t="inlineStr">
         <is>
-          <t>At the very least, Rurichiyo-chan is dreaming a gentle
-dream with pure feelings.</t>
+          <t>At the very least, Rurichiyo-chan is dreaming a
+gentle dream with pure feelings.</t>
         </is>
       </c>
       <c r="C948" t="n">
@@ -15080,8 +15095,8 @@
       </c>
       <c r="B951" s="1" t="inlineStr">
         <is>
-          <t>Above all, even if it was just a dream, Rurichiyo-chan
-was determined to do it.</t>
+          <t>Above all, even if it was just a dream,
+Rurichiyo-chan was determined to do it.</t>
         </is>
       </c>
       <c r="C951" t="n">
@@ -16523,8 +16538,8 @@
       </c>
       <c r="B1045" s="1" t="inlineStr">
         <is>
-          <t>「Aah... nfa...！ Sucking my boobs so much... good girl,
-dechu~... nfufu！」</t>
+          <t>「Aah... nfa...！ Sucking my boobs so much... good
+girl, dechu~... nfufu！」</t>
         </is>
       </c>
       <c r="C1045" t="n">
@@ -16539,8 +16554,8 @@
       </c>
       <c r="B1046" s="1" t="inlineStr">
         <is>
-          <t>Rurichiyo-chan’s dream is just of soothing a baby — an
-utterly innocent thing.</t>
+          <t>Rurichiyo-chan’s dream is just of soothing a baby —
+an utterly innocent thing.</t>
         </is>
       </c>
       <c r="C1046" t="n">
@@ -16555,8 +16570,8 @@
       </c>
       <c r="B1047" s="1" t="inlineStr">
         <is>
-          <t>And yet... bringing sexual desire into that feels like
-it would taint that purity.</t>
+          <t>And yet... bringing sexual desire into that feels
+like it would taint that purity.</t>
         </is>
       </c>
       <c r="C1047" t="n">
@@ -16804,7 +16819,8 @@
       </c>
       <c r="B1063" s="1" t="inlineStr">
         <is>
-          <t>Whoa... just thinking about it gets me so fired up...！</t>
+          <t>Whoa... just thinking about it gets me so fired
+up...！</t>
         </is>
       </c>
       <c r="C1063" t="n">
@@ -17065,8 +17081,8 @@
       </c>
       <c r="B1080" s="1" t="inlineStr">
         <is>
-          <t>…Reacting to Rurichiyo-chan's lustful voice, I too was
-overwhelmed.</t>
+          <t>…Reacting to Rurichiyo-chan's lustful voice, I too
+was overwhelmed.</t>
         </is>
       </c>
       <c r="C1080" t="n">
@@ -17959,9 +17975,9 @@
       <c r="B1138" s="1" t="inlineStr">
         <is>
           <t>I'm not doing anything wrong, so I could walk in
-confidently, but thinking about going to a girl's room
-this late at night brings along a certain kind of
-nervousness.</t>
+confidently, but thinking about going to a girl's
+room this late at night brings along a certain kind
+of nervousness.</t>
         </is>
       </c>
       <c r="C1138" t="n">
@@ -18009,8 +18025,8 @@
       </c>
       <c r="B1141" s="1" t="inlineStr">
         <is>
-          <t>No... but the purpose is strictly to just sleep beside
-her.</t>
+          <t>No... but the purpose is strictly to just sleep
+beside her.</t>
         </is>
       </c>
       <c r="C1141" t="n">
@@ -18240,8 +18256,8 @@
       </c>
       <c r="B1156" s="1" t="inlineStr">
         <is>
-          <t>A reasonable question, but kind of obvious on purpose,
-huh.</t>
+          <t>A reasonable question, but kind of obvious on
+purpose, huh.</t>
         </is>
       </c>
       <c r="C1156" t="n">
@@ -18486,7 +18502,8 @@
       </c>
       <c r="B1172" s="1" t="inlineStr">
         <is>
-          <t>...Alright, this calls for a straightforward approach.</t>
+          <t>...Alright, this calls for a straightforward
+approach.</t>
         </is>
       </c>
       <c r="C1172" t="n">
@@ -18730,8 +18747,8 @@
       </c>
       <c r="B1188" s="1" t="inlineStr">
         <is>
-          <t>It's painfully obvious, but maybe I shouldn't push her
-any further.</t>
+          <t>It's painfully obvious, but maybe I shouldn't push
+her any further.</t>
         </is>
       </c>
       <c r="C1188" t="n">
@@ -18746,8 +18763,8 @@
       </c>
       <c r="B1189" s="1" t="inlineStr">
         <is>
-          <t>I get it. If I go out of my way to flaunt that I know,
-she might end up hating me.</t>
+          <t>I get it. If I go out of my way to flaunt that I
+know, she might end up hating me.</t>
         </is>
       </c>
       <c r="C1189" t="n">
@@ -18962,8 +18979,8 @@
       <c r="B1203" s="1" t="inlineStr">
         <is>
           <t>「Um... could you sleep beside me... I mean, before
-going to sleep, do something like what Mom always used
-to do...」</t>
+going to sleep, do something like what Mom always
+used to do...」</t>
         </is>
       </c>
       <c r="C1203" t="n">
@@ -19070,7 +19087,8 @@
       </c>
       <c r="B1210" s="1" t="inlineStr">
         <is>
-          <t>When I answer honestly, Nono-chan nods as if relieved.</t>
+          <t>When I answer honestly, Nono-chan nods as if
+relieved.</t>
         </is>
       </c>
       <c r="C1210" t="n">
@@ -19524,8 +19542,8 @@
       </c>
       <c r="B1240" s="1" t="inlineStr">
         <is>
-          <t>By the way, my room used to be a closet, but it's also
-the highest room, so it has a great view.</t>
+          <t>By the way, my room used to be a closet, but it's
+also the highest room, so it has a great view.</t>
         </is>
       </c>
       <c r="C1240" t="n">
@@ -19650,8 +19668,8 @@
       </c>
       <c r="B1248" s="1" t="inlineStr">
         <is>
-          <t>Nono-chan mumbled and stumbled over her words, failing
-to get her point across.</t>
+          <t>Nono-chan mumbled and stumbled over her words,
+failing to get her point across.</t>
         </is>
       </c>
       <c r="C1248" t="n">
@@ -19865,8 +19883,9 @@
       </c>
       <c r="B1262" s="1" t="inlineStr">
         <is>
-          <t>「Actually, once I fall asleep, I don't seem to wake up
-easily, so I might end up causing you some trouble...」</t>
+          <t>「Actually, once I fall asleep, I don't seem to wake
+up easily, so I might end up causing you some
+trouble...」</t>
         </is>
       </c>
       <c r="C1262" t="n">
@@ -20823,8 +20842,8 @@
       </c>
       <c r="B1325" s="1" t="inlineStr">
         <is>
-          <t>「B-but. If you do the same thing you always do for me,
-I think I can sleep！」</t>
+          <t>「B-but. If you do the same thing you always do for
+me, I think I can sleep！」</t>
         </is>
       </c>
       <c r="C1325" t="n">
@@ -20855,8 +20874,8 @@
       </c>
       <c r="B1327" s="1" t="inlineStr">
         <is>
-          <t>The situation was moving so fast my head couldn’t keep
-up in places… but I understood.</t>
+          <t>The situation was moving so fast my head couldn’t
+keep up in places… but I understood.</t>
         </is>
       </c>
       <c r="C1327" t="n">
@@ -20993,8 +21012,8 @@
       </c>
       <c r="B1336" s="1" t="inlineStr">
         <is>
-          <t>Nono-chan was probably more worried about being unable
-to sleep than I had thought.</t>
+          <t>Nono-chan was probably more worried about being
+unable to sleep than I had thought.</t>
         </is>
       </c>
       <c r="C1336" t="n">
@@ -21669,8 +21688,8 @@
       <c r="B1380" s="1" t="inlineStr">
         <is>
           <t>And yet needing someone to sleep next to her would
-make her look like a little kid, and she wouldn't want
-everyone to know that.</t>
+make her look like a little kid, and she wouldn't
+want everyone to know that.</t>
         </is>
       </c>
       <c r="C1380" t="n">
@@ -22591,8 +22610,8 @@
       </c>
       <c r="B1440" s="1" t="inlineStr">
         <is>
-          <t>When I reached out to pick her up in a princess carry,
-I suddenly realized something.</t>
+          <t>When I reached out to pick her up in a princess
+carry, I suddenly realized something.</t>
         </is>
       </c>
       <c r="C1440" t="n">
@@ -22699,8 +22718,8 @@
       <c r="B1447" s="1" t="inlineStr">
         <is>
           <t>But given the situation—there's a girl asleep on the
-bed in my room... it would be strange not to be turned
-on.</t>
+bed in my room... it would be strange not to be
+turned on.</t>
         </is>
       </c>
       <c r="C1447" t="n">
@@ -22715,8 +22734,8 @@
       </c>
       <c r="B1448" s="1" t="inlineStr">
         <is>
-          <t>No, still, absentmindedly undoing the buttons can only
-be described as losing my mind.</t>
+          <t>No, still, absentmindedly undoing the buttons can
+only be described as losing my mind.</t>
         </is>
       </c>
       <c r="C1448" t="n">
@@ -22839,7 +22858,8 @@
       </c>
       <c r="B1456" s="1" t="inlineStr">
         <is>
-          <t>I snapped back to myself and shook my head in a panic.</t>
+          <t>I snapped back to myself and shook my head in a
+panic.</t>
         </is>
       </c>
       <c r="C1456" t="n">
@@ -23146,7 +23166,8 @@
       </c>
       <c r="B1476" s="1" t="inlineStr">
         <is>
-          <t>I wanted, at this point, to just strip her completely！</t>
+          <t>I wanted, at this point, to just strip her
+completely！</t>
         </is>
       </c>
       <c r="C1476" t="n">
@@ -23208,8 +23229,8 @@
       </c>
       <c r="B1480" s="1" t="inlineStr">
         <is>
-          <t>Even though it's my own hand, it feels like some other
-girl is stroking me.</t>
+          <t>Even though it's my own hand, it feels like some
+other girl is stroking me.</t>
         </is>
       </c>
       <c r="C1480" t="n">
@@ -23702,7 +23723,8 @@
       </c>
       <c r="B1512" s="1" t="inlineStr">
         <is>
-          <t>As expected, Nono-chan shows no sign of waking at all.</t>
+          <t>As expected, Nono-chan shows no sign of waking at
+all.</t>
         </is>
       </c>
       <c r="C1512" t="n">
@@ -23808,8 +23830,8 @@
       </c>
       <c r="B1519" s="1" t="inlineStr">
         <is>
-          <t>I wrap my palm in a slightly larger wad of tissues and
-wipe the semen off her cheek.</t>
+          <t>I wrap my palm in a slightly larger wad of tissues
+and wipe the semen off her cheek.</t>
         </is>
       </c>
       <c r="C1519" t="n">
@@ -24161,8 +24183,8 @@
       </c>
       <c r="B1542" s="1" t="inlineStr">
         <is>
-          <t>Maybe feeling something off at that spot, her sleeping
-breaths grow uneven.</t>
+          <t>Maybe feeling something off at that spot, her
+sleeping breaths grow uneven.</t>
         </is>
       </c>
       <c r="C1542" t="n">
@@ -24392,8 +24414,8 @@
       </c>
       <c r="B1557" s="1" t="inlineStr">
         <is>
-          <t>When the towel touched her chest, her sleeping breaths
-grew even more ragged.</t>
+          <t>When the towel touched her chest, her sleeping
+breaths grew even more ragged.</t>
         </is>
       </c>
       <c r="C1557" t="n">
@@ -24500,8 +24522,8 @@
       </c>
       <c r="B1564" s="1" t="inlineStr">
         <is>
-          <t>Sorry... this isn't the time to be enjoying myself, is
-it...</t>
+          <t>Sorry... this isn't the time to be enjoying myself,
+is it...</t>
         </is>
       </c>
       <c r="C1564" t="n">
@@ -24653,8 +24675,8 @@
       </c>
       <c r="B1574" s="1" t="inlineStr">
         <is>
-          <t>If I leave her alone, Nono-chan's breathing returns to
-normal, her breaths deepening.</t>
+          <t>If I leave her alone, Nono-chan's breathing returns
+to normal, her breaths deepening.</t>
         </is>
       </c>
       <c r="C1574" t="n">
@@ -24746,8 +24768,8 @@
       </c>
       <c r="B1580" s="1" t="inlineStr">
         <is>
-          <t>Come to think of it, even if she's a deep sleeper, she
-looks awfully quiet when she sleeps.</t>
+          <t>Come to think of it, even if she's a deep sleeper,
+she looks awfully quiet when she sleeps.</t>
         </is>
       </c>
       <c r="C1580" t="n">
@@ -24856,9 +24878,9 @@
       <c r="B1587" s="1" t="inlineStr">
         <is>
           <t>If the goal is for her to relax, it'd still be better
-if she slept here, but if that happens she'll probably
-feel awkward afterward, Nono-chan would try to be
-considerate.</t>
+if she slept here, but if that happens she'll
+probably feel awkward afterward, Nono-chan would try
+to be considerate.</t>
         </is>
       </c>
       <c r="C1587" t="n">

</xml_diff>